<commit_message>
Update chip report site 2026-06-17
</commit_message>
<xml_diff>
--- a/outputs/chip-report/台股盤後籌碼_2026-06-17.xlsx
+++ b/outputs/chip-report/台股盤後籌碼_2026-06-17.xlsx
@@ -1059,7 +1059,7 @@
       <c r="F40" s="6" t="n"/>
       <c r="G40" s="6" t="n"/>
       <c r="I40" s="6" t="n">
-        <v>0</v>
+        <v>25088</v>
       </c>
       <c r="J40" s="6" t="n"/>
       <c r="K40" s="6" t="n"/>
@@ -1092,7 +1092,7 @@
       <c r="G42" s="7" t="n"/>
       <c r="I42" s="7" t="inlineStr">
         <is>
-          <t>-67,849.70 - (-67,850) ≈ 0</t>
+          <t>|-67,849.70| - |-42,762| ≈ 25,088；結算日基準 5/20</t>
         </is>
       </c>
       <c r="J42" s="7" t="n"/>
@@ -1220,7 +1220,7 @@
     </row>
     <row r="52">
       <c r="A52" s="6" t="n">
-        <v>0</v>
+        <v>-815535</v>
       </c>
       <c r="B52" s="6" t="n"/>
       <c r="C52" s="6" t="n"/>
@@ -1249,7 +1249,7 @@
     <row r="54">
       <c r="A54" s="7" t="inlineStr">
         <is>
-          <t>408,477 - 408,477(6/17結算日 BC 原始金額)</t>
+          <t>408,477 - 1,224,012(5/20結算日 BC 原始金額)</t>
         </is>
       </c>
       <c r="B54" s="7" t="n"/>
@@ -1305,7 +1305,7 @@
     </row>
     <row r="58" ht="22" customHeight="1">
       <c r="A58" s="6" t="n">
-        <v>0</v>
+        <v>-83975</v>
       </c>
       <c r="B58" s="6" t="n"/>
       <c r="C58" s="6" t="n"/>
@@ -1334,7 +1334,7 @@
     <row r="60">
       <c r="A60" s="7" t="inlineStr">
         <is>
-          <t>323,784 - 323,784(6/17結算日 BP 原始金額)</t>
+          <t>323,784 - 407,759(5/20結算日 BP 原始金額)</t>
         </is>
       </c>
       <c r="B60" s="7" t="n"/>
@@ -1505,7 +1505,7 @@
       <c r="F72" s="6" t="n"/>
       <c r="G72" s="6" t="n"/>
       <c r="I72" s="6" t="n">
-        <v>0</v>
+        <v>-129816</v>
       </c>
       <c r="J72" s="6" t="n"/>
       <c r="K72" s="6" t="n"/>
@@ -1538,7 +1538,7 @@
       <c r="G74" s="7" t="n"/>
       <c r="I74" s="7" t="inlineStr">
         <is>
-          <t>889,709 - 889,709(6/17結算日 BC 原始金額)</t>
+          <t>889,709 - 1,019,525(5/20結算日 BC 原始金額)</t>
         </is>
       </c>
       <c r="J74" s="7" t="n"/>
@@ -1590,7 +1590,7 @@
       <c r="F78" s="6" t="n"/>
       <c r="G78" s="6" t="n"/>
       <c r="I78" s="6" t="n">
-        <v>0</v>
+        <v>-96761</v>
       </c>
       <c r="J78" s="6" t="n"/>
       <c r="K78" s="6" t="n"/>
@@ -1623,7 +1623,7 @@
       <c r="G80" s="7" t="n"/>
       <c r="I80" s="7" t="inlineStr">
         <is>
-          <t>260,937 - 260,937(6/17結算日 BP 原始金額)</t>
+          <t>260,937 - 357,698(5/20結算日 BP 原始金額)</t>
         </is>
       </c>
       <c r="J80" s="7" t="n"/>
@@ -1929,7 +1929,7 @@
     <row r="110">
       <c r="A110" s="16" t="inlineStr">
         <is>
-          <t>這是 2026-06-17 的盤後籌碼正式版：加權指數收 45,877.39 點、漲 68.20 點，盤中最高 45,877.39 點、最低 45,159.51 點，成交值約 11,545.96 億元；TWSE 信用交易統計已補回，融資金額餘額 5,839.12 億、較前一交易日增加 126.04 億，融券餘額 191,375 張、較前一交易日減少 3,150 張。TAIFEX 的外資(大小台)期貨未平倉依原表合併口徑 = TXF + MXF/4 + TMF/20，6/17 約為 -67,850，與結算比約 0、與前日增減約 854；主表 OP 欄位維持 BC-SC 與 BP-SP 的淨額口徑。</t>
+          <t>這是 2026-06-17 的盤後籌碼正式版：加權指數收 45,877.39 點、漲 68.20 點，盤中最高 45,877.39 點、最低 45,159.51 點，成交值約 11,545.96 億元；TWSE 信用交易統計已補回，融資金額餘額 5,839.12 億、較前一交易日增加 126.04 億，融券餘額 191,375 張、較前一交易日減少 3,150 張。TAIFEX 的外資(大小台)期貨未平倉依原表合併口徑 = TXF + MXF/4 + TMF/20，6/17 約為 -67,850，與結算比約 25,088、與前日增減約 854；主表 OP 欄位維持 BC-SC 與 BP-SP 的淨額口徑。</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update chip report site 2026-06-18
</commit_message>
<xml_diff>
--- a/outputs/chip-report/台股盤後籌碼_2026-06-17.xlsx
+++ b/outputs/chip-report/台股盤後籌碼_2026-06-17.xlsx
@@ -1041,7 +1041,8 @@
       <c r="G39" s="11" t="n"/>
       <c r="I39" s="11" t="inlineStr">
         <is>
-          <t>外資期貨未平倉與結算比</t>
+          <t>【SETTLE DAY】
+外資期貨未平倉與結算比</t>
         </is>
       </c>
       <c r="J39" s="11" t="n"/>
@@ -1092,7 +1093,7 @@
       <c r="G42" s="7" t="n"/>
       <c r="I42" s="7" t="inlineStr">
         <is>
-          <t>|-67,849.70| - |-42,762| ≈ 25,088；結算日基準 5/20</t>
+          <t>|-67,849.70| - |-42,762| ≈ 25,088；結算日基準 5/20；當日為結算日，本欄改以前次結算日 5/20 為基準。</t>
         </is>
       </c>
       <c r="J42" s="7" t="n"/>
@@ -1198,7 +1199,8 @@
     <row r="51">
       <c r="A51" s="11" t="inlineStr">
         <is>
-          <t>外資(BC)OP未平倉金額與結算比</t>
+          <t>【SETTLE DAY】
+外資(BC)OP未平倉金額與結算比</t>
         </is>
       </c>
       <c r="B51" s="11" t="n"/>
@@ -1249,7 +1251,7 @@
     <row r="54">
       <c r="A54" s="7" t="inlineStr">
         <is>
-          <t>408,477 - 1,224,012(5/20結算日 BC 原始金額)</t>
+          <t>408,477 - 1,224,012(5/20結算日 BC 原始金額)；當日為結算日，本欄改以前次結算日 5/20 為基準。</t>
         </is>
       </c>
       <c r="B54" s="7" t="n"/>
@@ -1283,7 +1285,8 @@
     <row r="57">
       <c r="A57" s="11" t="inlineStr">
         <is>
-          <t>外資(BP)OP未平倉金額與結算比</t>
+          <t>【SETTLE DAY】
+外資(BP)OP未平倉金額與結算比</t>
         </is>
       </c>
       <c r="B57" s="11" t="n"/>
@@ -1334,7 +1337,7 @@
     <row r="60">
       <c r="A60" s="7" t="inlineStr">
         <is>
-          <t>323,784 - 407,759(5/20結算日 BP 原始金額)</t>
+          <t>323,784 - 407,759(5/20結算日 BP 原始金額)；當日為結算日，本欄改以前次結算日 5/20 為基準。</t>
         </is>
       </c>
       <c r="B60" s="7" t="n"/>
@@ -1487,7 +1490,8 @@
       <c r="G71" s="13" t="n"/>
       <c r="I71" s="13" t="inlineStr">
         <is>
-          <t>自營(BC)OP未平倉金額與結算比</t>
+          <t>【SETTLE DAY】
+自營(BC)OP未平倉金額與結算比</t>
         </is>
       </c>
       <c r="J71" s="13" t="n"/>
@@ -1538,7 +1542,7 @@
       <c r="G74" s="7" t="n"/>
       <c r="I74" s="7" t="inlineStr">
         <is>
-          <t>889,709 - 1,019,525(5/20結算日 BC 原始金額)</t>
+          <t>889,709 - 1,019,525(5/20結算日 BC 原始金額)；當日為結算日，本欄改以前次結算日 5/20 為基準。</t>
         </is>
       </c>
       <c r="J74" s="7" t="n"/>
@@ -1572,7 +1576,8 @@
       <c r="G77" s="13" t="n"/>
       <c r="I77" s="13" t="inlineStr">
         <is>
-          <t>自營(BP)OP未平倉金額與結算比</t>
+          <t>【SETTLE DAY】
+自營(BP)OP未平倉金額與結算比</t>
         </is>
       </c>
       <c r="J77" s="13" t="n"/>
@@ -1623,7 +1628,7 @@
       <c r="G80" s="7" t="n"/>
       <c r="I80" s="7" t="inlineStr">
         <is>
-          <t>260,937 - 357,698(5/20結算日 BP 原始金額)</t>
+          <t>260,937 - 357,698(5/20結算日 BP 原始金額)；當日為結算日，本欄改以前次結算日 5/20 為基準。</t>
         </is>
       </c>
       <c r="J80" s="7" t="n"/>

</xml_diff>